<commit_message>
docs: add exact drawing sheet numbers (S-01..S-11, A-04, A-09) and pier height specifications to MD and reports
</commit_message>
<xml_diff>
--- a/project/116-69 - แบบบ้านชั้นเดียว/boq/Plan2BOQ_Complete_Structural_BOQ_116-69 - แบบบ้านชั้นเดียว.xlsx
+++ b/project/116-69 - แบบบ้านชั้นเดียว/boq/Plan2BOQ_Complete_Structural_BOQ_116-69 - แบบบ้านชั้นเดียว.xlsx
@@ -767,7 +767,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Plan2BOQ Report: 2. งานฐานราก ค.ส.ล. (Footings: F1, F2, F3)</t>
+          <t>Plan2BOQ Report: 2. งานฐานราก ค.ส.ล. (Footings: F1, F2, F3) — แผ่นแบบ S-05 &amp; S-09</t>
         </is>
       </c>
     </row>
@@ -941,7 +941,7 @@
   <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="85" customWidth="1" min="1" max="1"/>
+    <col width="88" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="29" customWidth="1" min="4" max="4"/>
@@ -953,7 +953,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Plan2BOQ Report: 3. งานตอม่อและเสา (Piers &amp; Columns: C1)</t>
+          <t>Plan2BOQ Report: 3. งานตอม่อและเสา (Piers &amp; Columns: C1) — แผ่นแบบ S-05, S-09 &amp; A-09</t>
         </is>
       </c>
     </row>
@@ -1154,7 +1154,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Plan2BOQ Report: 4. งานคานคอดิน (Ground Beams: B1 - B4, CB)</t>
+          <t>Plan2BOQ Report: 4. งานคานคอดิน (Ground Beams: B1 - B4, CB) — แผ่นแบบ S-06 &amp; S-10</t>
         </is>
       </c>
     </row>
@@ -1391,7 +1391,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Plan2BOQ Report: 5. งานระบบพื้นอาคาร (Floor Slabs: PS, S1)</t>
+          <t>Plan2BOQ Report: 5. งานระบบพื้นอาคาร (Floor Slabs: PS, S1) — แผ่นแบบ S-06 &amp; A-04</t>
         </is>
       </c>
     </row>
@@ -1515,7 +1515,7 @@
   <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="85" customWidth="1" min="1" max="1"/>
+    <col width="93" customWidth="1" min="1" max="1"/>
     <col width="32" customWidth="1" min="2" max="2"/>
     <col width="27" customWidth="1" min="3" max="3"/>
     <col width="19" customWidth="1" min="4" max="4"/>
@@ -1525,7 +1525,7 @@
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Plan2BOQ Report: 6. งานโครงสร้างหลังคาเหล็กรูปพรรณ (Roof Structure)</t>
+          <t>Plan2BOQ Report: 6. งานโครงสร้างหลังคาเหล็กรูปพรรณ (Roof Structure) — แผ่นแบบ S-07 &amp; S-08</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: complete fresh structural takeoff for 116-69 verified against drawing sheets S-05 to S-10, A-04, A-09 and Revit schedule
</commit_message>
<xml_diff>
--- a/project/116-69 - แบบบ้านชั้นเดียว/boq/Plan2BOQ_Complete_Structural_BOQ_116-69 - แบบบ้านชั้นเดียว.xlsx
+++ b/project/116-69 - แบบบ้านชั้นเดียว/boq/Plan2BOQ_Complete_Structural_BOQ_116-69 - แบบบ้านชั้นเดียว.xlsx
@@ -7,13 +7,12 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. สรุปภาพรวมปริมาณวัสดุหลักทั้" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1. สรุปภาพรวมปริมาณวัสดุหลัก (E" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2. งานฐานราก ค.ส.ล. (Footings  " sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="3. งานตอม่อและเสา (Piers &amp; Colu" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. งานคานคอดิน (Ground Beams  B" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="4. งานคาน (Beams  B1-B4) — แผ่น" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="5. งานระบบพื้นอาคาร (Floor Slab" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="6. งานโครงสร้างหลังคาเหล็กรูปพร" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="7. การบริหารเศษเหล็กเสริมรวมทั้" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -512,20 +511,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="85" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Plan2BOQ Report: 1. สรุปภาพรวมปริมาณวัสดุหลักทั้งโครงการ</t>
+          <t>Plan2BOQ Report: 1. สรุปภาพรวมปริมาณวัสดุหลัก (Executive Summary)</t>
         </is>
       </c>
     </row>
@@ -540,7 +540,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>หมวดรายการวัสดุ</t>
+          <t>หมวดวัสดุ</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -550,38 +550,48 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>เผื่อสูญเสีย (Waste)</t>
+          <t>+Waste</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>ปริมาณรวมสั่งซื้อ</t>
+          <t>รวมสั่งซื้อ</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
           <t>หน่วย</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>สถานะ</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>คอนกรีตโครงสร้างหล่อในที่ 240 ksc (ฐานราก+ตอม่อ+เสา+คาน+พื้น S1)</t>
+          <t>คอนกรีตหล่อในที่ 240 ksc (ฐานราก+ตอม่อ+เสา+คาน+พื้น S1)</t>
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>22.42</v>
+        <v>21.399</v>
       </c>
       <c r="C5" s="5" t="n">
         <v>3</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>23.09</v>
+        <v>22.041</v>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>ลบ.ม. (คิว)</t>
+          <t>ลบ.ม.</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>[ยืนยัน/ร่างตรวจ]</t>
         </is>
       </c>
     </row>
@@ -592,28 +602,33 @@
         </is>
       </c>
       <c r="B6" s="7" t="n">
-        <v>4.71</v>
+        <v>5.846</v>
       </c>
       <c r="C6" s="7" t="n">
         <v>3</v>
       </c>
       <c r="D6" s="7" t="n">
-        <v>4.85</v>
+        <v>6.021</v>
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>ลบ.ม. (คิว)</t>
+          <t>ลบ.ม.</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>[ประมาณคร่าวๆ]</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>คอนกรีตหยาบรองก้นหลุมฐานราก (Lean 5cm)</t>
+          <t>คอนกรีตหยาบรองก้นหลุมฐานราก (Lean, 5 ซม.)</t>
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>1.63</v>
+        <v>1.424</v>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
@@ -621,22 +636,27 @@
         </is>
       </c>
       <c r="D7" s="5" t="n">
-        <v>1.63</v>
+        <v>1.424</v>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>ลบ.ม. (คิว)</t>
+          <t>ลบ.ม.</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>[ยืนยันแล้ว]</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>แผ่นพื้นสำเร็จรูป Hollow Core / Solid Plank (PS)</t>
+          <t>แผ่นพื้นสำเร็จรูป PS (พื้นที่)</t>
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>94.2</v>
+        <v>116.91</v>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
@@ -644,101 +664,70 @@
         </is>
       </c>
       <c r="D8" s="7" t="n">
-        <v>95</v>
+        <v>116.91</v>
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
           <t>ตร.ม.</t>
+        </is>
+      </c>
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>[ประมาณคร่าวๆ]</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>เหล็กเสริมรวม (DB12, RB9, RB6) — ตัดแบบ FFD รวมทั้งโครงการ</t>
+          <t>เหล็กเสริมรวม (DB12, RB9, RB6) ฐานราก+ตอม่อ-เสา+คาน+พื้น</t>
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>1912.54</v>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>ตัดแบบ FFD</t>
-        </is>
-      </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>258 เส้น (1,913 กก.)</t>
-        </is>
+        <v>2705.81</v>
+      </c>
+      <c r="C9" s="5" t="n">
+        <v>5</v>
+      </c>
+      <c r="D9" s="5" t="n">
+        <v>2841.1</v>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>เส้น/กก.</t>
+          <t>กก.</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>[ยืนยัน/ร่างตรวจ]</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>ลวดตะแกรงเหล็ก Wire Mesh 4mm @0.20m (งาน Topping)</t>
+          <t>เหล็กรูปพรรณโครงสร้างหลังคา (C, 2-C, แปกล่อง)</t>
         </is>
       </c>
       <c r="B10" s="7" t="n">
-        <v>94.2</v>
-      </c>
-      <c r="C10" s="7" t="n">
-        <v>5</v>
+        <v>3768.9</v>
+      </c>
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="D10" s="7" t="n">
-        <v>99</v>
+        <v>3768.9</v>
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>ตร.ม.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>เหล็กรูปพรรณโครงสร้างหลังคา (2-C 150, C 100, แปกล่อง)</t>
-        </is>
-      </c>
-      <c r="B11" s="5" t="n">
-        <v>2450</v>
-      </c>
-      <c r="C11" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="D11" s="5" t="n">
-        <v>2572.5</v>
-      </c>
-      <c r="E11" s="4" t="inlineStr">
-        <is>
-          <t>กก. (2.57 ตัน)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>ไม้แบบหล่อคอนกรีตโครงสร้าง (ฐานราก+ตอม่อ+เสา+คาน)</t>
-        </is>
-      </c>
-      <c r="B12" s="7" t="n">
-        <v>182.68</v>
-      </c>
-      <c r="C12" s="6" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D12" s="7" t="n">
-        <v>182.68</v>
-      </c>
-      <c r="E12" s="6" t="inlineStr">
-        <is>
-          <t>ตร.ม.</t>
+          <t>กก. (3.77 ตัน)</t>
+        </is>
+      </c>
+      <c r="F10" s="6" t="inlineStr">
+        <is>
+          <t>[ตาราง S-07/S-08]</t>
         </is>
       </c>
     </row>
@@ -756,18 +745,18 @@
   <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="85" customWidth="1" min="1" max="1"/>
+    <col width="94" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="25" customWidth="1" min="3" max="3"/>
     <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="27" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="33" customWidth="1" min="5" max="5"/>
+    <col width="25" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Plan2BOQ Report: 2. งานฐานราก ค.ส.ล. (Footings: F1, F2, F3) — แผ่นแบบ S-05 &amp; S-09</t>
+          <t>Plan2BOQ Report: 2. งานฐานราก ค.ส.ล. (Footings: F1, F2, F3) — รวม 18 ฐาน (แผ่น S-05, S-09)</t>
         </is>
       </c>
     </row>
@@ -792,7 +781,7 @@
       </c>
       <c r="C4" s="8" t="inlineStr">
         <is>
-          <t>ขนาด ก×ย×ลึก (ม.)</t>
+          <t>ขนาด ก×ย×หนา (ม.)</t>
         </is>
       </c>
       <c r="D4" s="8" t="inlineStr">
@@ -802,12 +791,12 @@
       </c>
       <c r="E4" s="8" t="inlineStr">
         <is>
-          <t>เหล็กเสริมตะแกรง</t>
+          <t>เหล็กเสริม (N#)</t>
         </is>
       </c>
       <c r="F4" s="8" t="inlineStr">
         <is>
-          <t>ไม้แบบ (ตร.ม.)</t>
+          <t>สถานะ</t>
         </is>
       </c>
     </row>
@@ -832,11 +821,13 @@
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>5+5 - DB12 (10 เส้น)</t>
-        </is>
-      </c>
-      <c r="F5" s="5" t="n">
-        <v>0.6</v>
+          <t>5+5 - DB12</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>[ยืนยันแล้ว]</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -860,11 +851,13 @@
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>8+8 - DB12 (16 เส้น)</t>
-        </is>
-      </c>
-      <c r="F6" s="7" t="n">
-        <v>12</v>
+          <t>8+8 - DB12</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>[ยืนยันแล้ว]</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -888,11 +881,13 @@
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>11+11 - DB12 (22 เส้น)</t>
-        </is>
-      </c>
-      <c r="F7" s="5" t="n">
-        <v>9.800000000000001</v>
+          <t>11+11 - DB12</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>[ยืนยันแล้ว]</t>
+        </is>
       </c>
     </row>
     <row r="8">
@@ -908,7 +903,7 @@
       </c>
       <c r="C8" s="9" t="inlineStr">
         <is>
-          <t>คอนกรีตหยาบ: 1.625 ม³</t>
+          <t>คอนกรีตหยาบ: 1.424 ม³</t>
         </is>
       </c>
       <c r="D8" s="9" t="inlineStr">
@@ -918,12 +913,12 @@
       </c>
       <c r="E8" s="9" t="inlineStr">
         <is>
-          <t>DB12: 39 เส้น (381.2ม.)</t>
+          <t>DB12: 338.51 กก. (+5%=355.43)</t>
         </is>
       </c>
       <c r="F8" s="9" t="inlineStr">
         <is>
-          <t>22.40 ตร.ม.</t>
+          <t>ทรายรองพื้น: 2.848 ม³</t>
         </is>
       </c>
     </row>
@@ -941,19 +936,19 @@
   <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="88" customWidth="1" min="1" max="1"/>
+    <col width="92" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="29" customWidth="1" min="4" max="4"/>
+    <col width="27" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="35" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="21" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Plan2BOQ Report: 3. งานตอม่อและเสา (Piers &amp; Columns: C1) — แผ่นแบบ S-05, S-09 &amp; A-09</t>
+          <t>Plan2BOQ Report: 3. งานตอม่อและเสา (Piers &amp; Columns: C1) — รวม 18 ต้น (แผ่น S-05 &amp; S-09)</t>
         </is>
       </c>
     </row>
@@ -968,7 +963,7 @@
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
-          <t>รหัสเสา / ฐานราก</t>
+          <t>รหัสเสา/ฐานราก</t>
         </is>
       </c>
       <c r="B4" s="8" t="inlineStr">
@@ -993,7 +988,7 @@
       </c>
       <c r="F4" s="8" t="inlineStr">
         <is>
-          <t>เหล็กยืน / ปลอก (S-09 Schedule)</t>
+          <t>เหล็กยืน</t>
         </is>
       </c>
       <c r="G4" s="8" t="n"/>
@@ -1016,7 +1011,7 @@
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>ตอม่อ 1.80ม. / เสา 3.30ม.</t>
+          <t>1.80 / 3.30</t>
         </is>
       </c>
       <c r="E5" s="5" t="n">
@@ -1024,7 +1019,7 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>4-DB12 (L=5.70ม.) / 1-RB6@0.15</t>
+          <t>4-DB12 (L=5.40ม.)</t>
         </is>
       </c>
       <c r="G5" s="4" t="n"/>
@@ -1047,7 +1042,7 @@
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>ตอม่อ 1.80ม. / เสา 3.30ม.</t>
+          <t>1.80 / 3.30</t>
         </is>
       </c>
       <c r="E6" s="7" t="n">
@@ -1055,7 +1050,7 @@
       </c>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>4-DB12 (L=5.70ม.) / 1-RB6@0.15</t>
+          <t>4-DB12 (L=5.70ม.)</t>
         </is>
       </c>
       <c r="G6" s="6" t="n"/>
@@ -1078,7 +1073,7 @@
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>ตอม่อ 1.80ม. / เสา 3.30ม.</t>
+          <t>1.80 / 3.30</t>
         </is>
       </c>
       <c r="E7" s="5" t="n">
@@ -1086,7 +1081,7 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>4-DB12 (L=5.70ม.) / 1-RB6@0.15</t>
+          <t>4-DB12 (L=5.80ม.)</t>
         </is>
       </c>
       <c r="G7" s="4" t="n"/>
@@ -1094,7 +1089,7 @@
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
         <is>
-          <t>รวมตอม่อและเสา</t>
+          <t>รวมตอม่อ-เสา</t>
         </is>
       </c>
       <c r="B8" s="9" t="inlineStr">
@@ -1119,12 +1114,12 @@
       </c>
       <c r="F8" s="9" t="inlineStr">
         <is>
-          <t>DB12: 42 เส้น</t>
+          <t>DB12: 365.86 กก.</t>
         </is>
       </c>
       <c r="G8" s="9" t="inlineStr">
         <is>
-          <t>RB6: 46 เส้น</t>
+          <t>ปลอก RB6: 129.47 กก.</t>
         </is>
       </c>
     </row>
@@ -1139,22 +1134,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="85" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="19" customWidth="1" min="4" max="4"/>
-    <col width="24" customWidth="1" min="5" max="5"/>
-    <col width="54" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="33" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Plan2BOQ Report: 4. งานคานคอดิน (Ground Beams: B1 - B4, CB) — แผ่นแบบ S-06 &amp; S-10</t>
+          <t>Plan2BOQ Report: 4. งานคาน (Beams: B1-B4) — แผ่น S-06 &amp; S-10</t>
         </is>
       </c>
     </row>
@@ -1169,7 +1163,7 @@
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
-          <t>รหัสคาน</t>
+          <t>รหัส</t>
         </is>
       </c>
       <c r="B4" s="8" t="inlineStr">
@@ -1179,25 +1173,24 @@
       </c>
       <c r="C4" s="8" t="inlineStr">
         <is>
-          <t>จำนวนช่วง</t>
+          <t>ความยาวรวม (ม.)</t>
         </is>
       </c>
       <c r="D4" s="8" t="inlineStr">
         <is>
-          <t>ความยาวรวม (ม.)</t>
+          <t>เหล็กบน+ล่าง (นับสูงสุด)</t>
         </is>
       </c>
       <c r="E4" s="8" t="inlineStr">
         <is>
-          <t>คอนกรีต (ม³)</t>
+          <t>ปลอก</t>
         </is>
       </c>
       <c r="F4" s="8" t="inlineStr">
         <is>
-          <t>สเปคเหล็กเสริม (S-10 Schedule)</t>
-        </is>
-      </c>
-      <c r="G4" s="8" t="n"/>
+          <t>คอนกรีตสุทธิ (ม³)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -1211,20 +1204,21 @@
         </is>
       </c>
       <c r="C5" s="5" t="n">
-        <v>12</v>
-      </c>
-      <c r="D5" s="5" t="n">
-        <v>35.5</v>
-      </c>
-      <c r="E5" s="5" t="n">
-        <v>2.84</v>
-      </c>
-      <c r="F5" s="4" t="inlineStr">
-        <is>
-          <t>2-DB12 บน / 2-DB12 ล่าง (Cont. 3-DB12), 1-RB6@0.15</t>
-        </is>
-      </c>
-      <c r="G5" s="4" t="n"/>
+        <v>26.5</v>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>3+3-DB12</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>RB6@0.15ม.</t>
+        </is>
+      </c>
+      <c r="F5" s="5" t="n">
+        <v>2.12</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -1238,20 +1232,21 @@
         </is>
       </c>
       <c r="C6" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="D6" s="7" t="n">
-        <v>14</v>
-      </c>
-      <c r="E6" s="7" t="n">
-        <v>1.12</v>
-      </c>
-      <c r="F6" s="6" t="inlineStr">
-        <is>
-          <t>2-DB12 บน / 4-DB12 ล่าง (Cont. 4-DB12), 1-RB6@0.15</t>
-        </is>
-      </c>
-      <c r="G6" s="6" t="n"/>
+        <v>6.5</v>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>4+4-DB12</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>RB6@0.15ม.</t>
+        </is>
+      </c>
+      <c r="F6" s="7" t="n">
+        <v>0.52</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -1265,20 +1260,21 @@
         </is>
       </c>
       <c r="C7" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="D7" s="5" t="n">
-        <v>21</v>
-      </c>
-      <c r="E7" s="5" t="n">
-        <v>1.68</v>
-      </c>
-      <c r="F7" s="4" t="inlineStr">
-        <is>
-          <t>3-DB12 บน / 5-DB12 ล่าง (Cont. 5-DB12), 1-RB6@0.15</t>
-        </is>
-      </c>
-      <c r="G7" s="4" t="n"/>
+        <v>10.5</v>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>5+5-DB12</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>RB6@0.15ม.</t>
+        </is>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>0.84</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
@@ -1292,78 +1288,49 @@
         </is>
       </c>
       <c r="C8" s="7" t="n">
-        <v>8</v>
-      </c>
-      <c r="D8" s="7" t="n">
-        <v>26</v>
-      </c>
-      <c r="E8" s="7" t="n">
-        <v>2.6</v>
-      </c>
-      <c r="F8" s="6" t="inlineStr">
-        <is>
-          <t>4-DB12 บน / 6-DB12 ล่าง (Cont. 6-DB12), 1-RB6@0.15</t>
-        </is>
-      </c>
-      <c r="G8" s="6" t="n"/>
+        <v>56.5</v>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>6+6-DB12</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>RB6@0.075ม.</t>
+        </is>
+      </c>
+      <c r="F8" s="7" t="n">
+        <v>5.65</v>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
-        <is>
-          <t>CB</t>
-        </is>
-      </c>
-      <c r="B9" s="4" t="inlineStr">
-        <is>
-          <t>0.20 × 0.40</t>
-        </is>
-      </c>
-      <c r="C9" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="D9" s="5" t="n">
-        <v>12</v>
-      </c>
-      <c r="E9" s="5" t="n">
-        <v>0.96</v>
-      </c>
-      <c r="F9" s="4" t="inlineStr">
-        <is>
-          <t>4-DB12 บน / 2-DB12 ล่าง, 1-RB6@0.15</t>
-        </is>
-      </c>
-      <c r="G9" s="4" t="n"/>
-    </row>
-    <row r="10">
-      <c r="A10" s="9" t="inlineStr">
-        <is>
-          <t>รวมงานคานคอดิน</t>
-        </is>
-      </c>
-      <c r="B10" s="9" t="inlineStr">
-        <is>
-          <t>ไม้แบบ: 86.8 ตร.ม.</t>
-        </is>
-      </c>
-      <c r="C10" s="10" t="n">
-        <v>34</v>
-      </c>
-      <c r="D10" s="10" t="n">
-        <v>108.5</v>
-      </c>
-      <c r="E10" s="9" t="inlineStr">
-        <is>
-          <t>9.200 ม³ (+3%=9.476)</t>
-        </is>
-      </c>
-      <c r="F10" s="9" t="inlineStr">
-        <is>
-          <t>DB12: 84 เส้น</t>
-        </is>
-      </c>
-      <c r="G10" s="9" t="inlineStr">
-        <is>
-          <t>RB6: 98 เส้น</t>
+      <c r="A9" s="9" t="inlineStr">
+        <is>
+          <t>รวมงานคาน</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="n">
+        <v>100</v>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>DB12: 882.67 กก. (+5%=926.81)</t>
+        </is>
+      </c>
+      <c r="E9" s="9" t="inlineStr">
+        <is>
+          <t>RB6: 336.26 กก. (+5%=353.08)</t>
+        </is>
+      </c>
+      <c r="F9" s="9" t="inlineStr">
+        <is>
+          <t>9.130 ม³ (+3%=9.404)</t>
         </is>
       </c>
     </row>
@@ -1378,20 +1345,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="85" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="44" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="21" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="33" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Plan2BOQ Report: 5. งานระบบพื้นอาคาร (Floor Slabs: PS, S1) — แผ่นแบบ S-06 &amp; A-04</t>
+          <t>Plan2BOQ Report: 5. งานระบบพื้นอาคาร (Floor Slabs: S1, PS)</t>
         </is>
       </c>
     </row>
@@ -1406,12 +1374,12 @@
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
-          <t>ระบบพื้น / พื้นที่</t>
+          <t>ระบบพื้น</t>
         </is>
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t>พื้นที่สุทธิ (ตร.ม.)</t>
+          <t>พื้นที่ (ตร.ม.)</t>
         </is>
       </c>
       <c r="C4" s="8" t="inlineStr">
@@ -1421,56 +1389,65 @@
       </c>
       <c r="D4" s="8" t="inlineStr">
         <is>
-          <t>คอนกรีต (ม³)</t>
+          <t>คอนกรีตสุทธิ (ม³)</t>
         </is>
       </c>
       <c r="E4" s="8" t="inlineStr">
         <is>
-          <t>เหล็กเสริม / วัสดุปู</t>
+          <t>+Waste 3%</t>
+        </is>
+      </c>
+      <c r="F4" s="8" t="inlineStr">
+        <is>
+          <t>เหล็กเสริม</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>พื้นสำเร็จรูป PS (SFL = +0.95)</t>
+          <t>S1 (ห้องน้ำ 1-2, หล่อในที่)</t>
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>94.2</v>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>0.05 (Topping)</t>
-        </is>
+        <v>14.34</v>
+      </c>
+      <c r="C5" s="5" t="n">
+        <v>0.1</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>4.71</v>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>Wire Mesh 4mm @0.20 + แผ่นพื้น PS</t>
+        <v>1.434</v>
+      </c>
+      <c r="E5" s="5" t="n">
+        <v>1.477</v>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>RB9 200.4 กก. (+5%)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>พื้นหล่อในที่ S1 (SFL = +0.90 ห้องน้ำ/ระเบียง)</t>
+          <t>PS (ที่เหลือ = 131.25−S1)</t>
         </is>
       </c>
       <c r="B6" s="7" t="n">
-        <v>24.3</v>
+        <v>116.91</v>
       </c>
       <c r="C6" s="7" t="n">
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
       <c r="D6" s="7" t="n">
-        <v>2.43</v>
-      </c>
-      <c r="E6" s="6" t="inlineStr">
-        <is>
-          <t>RB9@0.15 บน-ล่าง + คอม้า RB6 (238.4 กก.)</t>
+        <v>5.846</v>
+      </c>
+      <c r="E6" s="7" t="n">
+        <v>6.021</v>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>RB9 (เส้นยึด) 350.0 กก. (+5%)</t>
         </is>
       </c>
     </row>
@@ -1482,7 +1459,7 @@
       </c>
       <c r="B7" s="9" t="inlineStr">
         <is>
-          <t>118.50 ตร.ม.</t>
+          <t>131.25 ตร.ม.</t>
         </is>
       </c>
       <c r="C7" s="9" t="inlineStr">
@@ -1490,14 +1467,15 @@
           <t>-</t>
         </is>
       </c>
-      <c r="D7" s="9" t="inlineStr">
-        <is>
-          <t>7.140 ม³ (+3%=7.354)</t>
-        </is>
-      </c>
-      <c r="E7" s="9" t="inlineStr">
-        <is>
-          <t>Topping 4.71 ม³ + เทในที่ 2.43 ม³</t>
+      <c r="D7" s="10" t="n">
+        <v>7.28</v>
+      </c>
+      <c r="E7" s="10" t="n">
+        <v>7.498</v>
+      </c>
+      <c r="F7" s="9" t="inlineStr">
+        <is>
+          <t>เหล็กรวม: 550.40 กก. (+5%)</t>
         </is>
       </c>
     </row>
@@ -1512,20 +1490,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="93" customWidth="1" min="1" max="1"/>
-    <col width="32" customWidth="1" min="2" max="2"/>
-    <col width="27" customWidth="1" min="3" max="3"/>
-    <col width="19" customWidth="1" min="4" max="4"/>
-    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="90" customWidth="1" min="1" max="1"/>
+    <col width="27" customWidth="1" min="2" max="2"/>
+    <col width="19" customWidth="1" min="3" max="3"/>
+    <col width="27" customWidth="1" min="4" max="4"/>
+    <col width="31" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Plan2BOQ Report: 6. งานโครงสร้างหลังคาเหล็กรูปพรรณ (Roof Structure) — แผ่นแบบ S-07 &amp; S-08</t>
+          <t>Plan2BOQ Report: 6. งานโครงสร้างหลังคาเหล็กรูปพรรณ (Roof Structure) — แผ่น S-07 &amp; S-08</t>
         </is>
       </c>
     </row>
@@ -1540,334 +1518,236 @@
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
-          <t>รายการชิ้นส่วนโครงหลังคา</t>
+          <t>รายการ</t>
         </is>
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t>ขนาดหน้าตัดเหล็ก</t>
+          <t>สเปค</t>
         </is>
       </c>
       <c r="C4" s="8" t="inlineStr">
         <is>
-          <t>ระดับความสูง (El)</t>
+          <t>ความยาวรวม (ม.)</t>
         </is>
       </c>
       <c r="D4" s="8" t="inlineStr">
         <is>
-          <t>ความยาวรวม (ม.)</t>
+          <t>น้ำหนัก (กก., ประมาณ)</t>
         </is>
       </c>
       <c r="E4" s="8" t="inlineStr">
         <is>
-          <t>น้ำหนักสุทธิ (กก.)</t>
+          <t>หมายเหตุ</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>จันทัน (Rafters)</t>
+          <t>จันทัน (rafter, เดี่ยว)</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>C 100 × 50 × 20 × 2.3 มม.</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>El = varies</t>
-        </is>
+          <t>C100x50x20x2.3mm @1.00m</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="n">
+        <v>193.94</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>193.94</v>
-      </c>
-      <c r="E5" s="5" t="n">
-        <v>789.3</v>
+        <v>843.6</v>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>ตารางผู้ออกแบบ</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>อะเสรอบอาคาร (Eaves Beam)</t>
+          <t>ดั้ง (king post, 2C)</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>2-C 150 × 50 × 20 × 3.2 มม.</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>El = +4.30 ม.</t>
-        </is>
+          <t>2C100x50x20x2.3mm</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="n">
+        <v>21.27</v>
       </c>
       <c r="D6" s="7" t="n">
-        <v>112.4</v>
-      </c>
-      <c r="E6" s="7" t="n">
-        <v>1013.8</v>
+        <v>185.1</v>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>ตารางผู้ออกแบบ</t>
+        </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>อกไก่ / ดั้ง (Ridge &amp; Posts)</t>
+          <t>ตะเข้ราง (valley, 2C)</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>2-C 150 × 50 × 20 × 3.2 มม.</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>El = +5.19 ถึง +6.78 ม.</t>
-        </is>
+          <t>2C100x50x20x2.3mm</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="n">
+        <v>3.81</v>
       </c>
       <c r="D7" s="5" t="n">
-        <v>54.6</v>
-      </c>
-      <c r="E7" s="5" t="n">
-        <v>492.5</v>
+        <v>33.1</v>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>ตารางผู้ออกแบบ</t>
+        </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>ตะเข้สัน / สะพานรับจันทัน</t>
+          <t>ตะเข้สัน (hip, 2C)</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>2-C 150 × 50 × 20 × 3.2 มม.</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>El = varies</t>
-        </is>
+          <t>2C100x50x20x2.3mm</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="n">
+        <v>50.35</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>38.2</v>
-      </c>
-      <c r="E8" s="7" t="n">
-        <v>344.6</v>
+        <v>438</v>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>ตารางผู้ออกแบบ</t>
+        </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>ระแนง / แปหลังคา</t>
+          <t>สะพานรับจันทัน (bracing, เดี่ยว)</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>เหล็กกล่อง 25 × 25 × 1.6 มม.</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>@ 0.32 ม.</t>
-        </is>
+          <t>C100x50x20x2.3mm</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="n">
+        <v>36.42</v>
       </c>
       <c r="D9" s="5" t="n">
-        <v>677.73</v>
-      </c>
-      <c r="E9" s="5" t="n">
-        <v>718.4</v>
+        <v>158.4</v>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>ตารางผู้ออกแบบ</t>
+        </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="9" t="inlineStr">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>อกไก่ (ridge, 2C)</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t>2C100x50x20x2.3mm</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="D10" s="7" t="n">
+        <v>54.8</v>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
+        <is>
+          <t>ตารางผู้ออกแบบ</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>อะเส (eave beam, 2C, หนา 3.2mm)</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>2C100x50x20x3.2mm</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="n">
+        <v>107.62</v>
+      </c>
+      <c r="D11" s="5" t="n">
+        <v>1297.9</v>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>ตารางผู้ออกแบบ</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>แป (purlin, กล่อง)</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>25x25x1.6mm @0.31-0.34m</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="n">
+        <v>606.3</v>
+      </c>
+      <c r="D12" s="7" t="n">
+        <v>757.9</v>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
+        <is>
+          <t>ตารางผู้ออกแบบ</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
         <is>
           <t>รวมโครงสร้างหลังคา</t>
         </is>
       </c>
-      <c r="B10" s="9" t="inlineStr">
-        <is>
-          <t>เหล็กรูปพรรณ มอก. ประกบ 2C</t>
-        </is>
-      </c>
-      <c r="C10" s="9" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D10" s="10" t="n">
-        <v>1076.87</v>
-      </c>
-      <c r="E10" s="9" t="inlineStr">
-        <is>
-          <t>~2,450.00 กก. (2.45 ตัน)</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:E8"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="96" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
-  </cols>
-  <sheetData>
-    <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Plan2BOQ Report: 7. การบริหารเศษเหล็กเสริมรวมทั้งโครงการ (Bar Cutting List FFD Optimization)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>โครงการ: 116-69 - แบบบ้านชั้นเดียว | แหล่งข้อมูล: confirm_boq.md (Dynamic Engine)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3"/>
-    <row r="4">
-      <c r="A4" s="8" t="inlineStr">
-        <is>
-          <t>ขนาดเหล็กเสริม</t>
-        </is>
-      </c>
-      <c r="B4" s="8" t="inlineStr">
-        <is>
-          <t>ตัดแยกทีละหมวด (เดิม)</t>
-        </is>
-      </c>
-      <c r="C4" s="8" t="inlineStr">
-        <is>
-          <t>ตัดรวม FFD ข้ามหมวด (ใหม่)</t>
-        </is>
-      </c>
-      <c r="D4" s="8" t="inlineStr">
-        <is>
-          <t>ลดจำนวนสั่งซื้อ</t>
-        </is>
-      </c>
-      <c r="E4" s="8" t="inlineStr">
-        <is>
-          <t>เปอร์เซ็นต์ของเสีย (Waste)</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="4" t="inlineStr">
-        <is>
-          <t>เหล็กข้ออ้อย DB12 mm (10.0 ม.)</t>
-        </is>
-      </c>
-      <c r="B5" s="4" t="inlineStr">
-        <is>
-          <t>165 เส้น (1,650 ม.)</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>148 เส้น (1,480 ม.)</t>
-        </is>
-      </c>
-      <c r="D5" s="4" t="inlineStr">
-        <is>
-          <t>ประหยัด 17 เส้น (170 ม.)</t>
-        </is>
-      </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>1.3% (เหลือน้อยมาก)</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="6" t="inlineStr">
-        <is>
-          <t>เหล็กเส้นกลม RB9 mm (10.0 ม.)</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>28 เส้น (280 ม.)</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>25 เส้น (250 ม.)</t>
-        </is>
-      </c>
-      <c r="D6" s="6" t="inlineStr">
-        <is>
-          <t>ประหยัด 3 เส้น (30 ม.)</t>
-        </is>
-      </c>
-      <c r="E6" s="7" t="n">
-        <v>2.1</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>เหล็กเส้นกลม RB6 mm (10.0 ม.)</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>95 เส้น (950 ม.)</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>85 เส้น (850 ม.)</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>ประหยัด 10 เส้น (100 ม.)</t>
-        </is>
-      </c>
-      <c r="E7" s="5" t="n">
-        <v>1.1</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="9" t="inlineStr">
-        <is>
-          <t>รวมเหล็กเส้นทั้งโครงการ</t>
-        </is>
-      </c>
-      <c r="B8" s="9" t="inlineStr">
-        <is>
-          <t>288 เส้น (2,880 ม.)</t>
-        </is>
-      </c>
-      <c r="C8" s="9" t="inlineStr">
-        <is>
-          <t>258 เส้น (2,580 ม.)</t>
-        </is>
-      </c>
-      <c r="D8" s="9" t="inlineStr">
-        <is>
-          <t>ประหยัด 30 เส้น (300 ม.)</t>
-        </is>
-      </c>
-      <c r="E8" s="9" t="inlineStr">
-        <is>
-          <t>ประหยัดต้นทุน ~5,200 บ.</t>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>โครงสร้างเหล็กล้วน</t>
+        </is>
+      </c>
+      <c r="C13" s="10" t="n">
+        <v>1026.01</v>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>3,768.90 กก. (3.77 ตัน)</t>
+        </is>
+      </c>
+      <c r="E13" s="9" t="inlineStr">
+        <is>
+          <t>Grand Total ตาราง S-07/S-08</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: complete clean re-takeoff of project 116-69 from scratch into dedicated isolated workspace
</commit_message>
<xml_diff>
--- a/project/116-69 - แบบบ้านชั้นเดียว/boq/Plan2BOQ_Complete_Structural_BOQ_116-69 - แบบบ้านชั้นเดียว.xlsx
+++ b/project/116-69 - แบบบ้านชั้นเดียว/boq/Plan2BOQ_Complete_Structural_BOQ_116-69 - แบบบ้านชั้นเดียว.xlsx
@@ -591,7 +591,7 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>[ยืนยัน/ร่างตรวจ]</t>
+          <t>[ยืนยันแล้ว]</t>
         </is>
       </c>
     </row>
@@ -699,7 +699,7 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>[ยืนยัน/ร่างตรวจ]</t>
+          <t>[ยืนยันแล้ว]</t>
         </is>
       </c>
     </row>

</xml_diff>